<commit_message>
Leads: 2026-10-23 13:19 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-23.xlsx
+++ b/output/leads_2026-10-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,66 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Montani Mechanical Group</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>plumbercharlestonwv.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.plumbercharlestonwv.com/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Greater Charleston</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>service@montanimg.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>(304) 220-0181</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Charleston WV</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>88</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>plumber Charleston WV</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-23 13:31 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-23.xlsx
+++ b/output/leads_2026-10-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,66 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>WY&amp;G, Inc. Heating and Air</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>wyginc.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.wyginc.com/heater-repair-palmdale/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Trade Show</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>info@wyginc.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(323) 240-2373</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Palmdale CA</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>90</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>furnace repair Palmdale CA</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-23 13:32 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-23.xlsx
+++ b/output/leads_2026-10-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Everett Metal Roofing Experts | Durable &amp; Energy-Efficient Roof Solutions</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>riversideroofingllc.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.riversideroofingllc.com/everett-metal-roofing</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Master Elite</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@riversideroofingllc.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(425) 949-8252</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Everett WA</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Everett WA</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-23 13:34 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-23.xlsx
+++ b/output/leads_2026-10-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -743,6 +743,186 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Clarksville Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>clarksvillecomfort.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://clarksvillecomfort.com/heating-and-air-conditioning-columbia-md/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Owner As</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>service@clarksvillecomfort.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>443-324-0728</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Columbia MD</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>air conditioning repair Columbia MD</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Heating &amp; Air Conditioning Columbia, MD | Lindy M. Redding HVAC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>lindyredding.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://www.lindyredding.com/columbia--md</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Maintenance Since</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>lmredding@verizon.net</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>410-987-4070</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Columbia MD</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>90</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>air conditioning repair Columbia MD</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Nichols Construction, LLC</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>nicholsconstructionllc.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://nicholsconstructionllc.com/service-areas/fayetteville-ar/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>When Fayetteville</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>info@nicholsconstructionllc.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(417) 250-1049</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Fayetteville AR</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>88</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Fayetteville AR</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-23 19:54 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-23.xlsx
+++ b/output/leads_2026-10-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -923,6 +923,126 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Roof United</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>roofbrokenarrow.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://roofbrokenarrow.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Claims Services</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>raf@roofunited.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>918-505-2335</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>roof replacement Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Roof Monster</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>roofmonster.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://roofmonster.com/orem/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Roof Monster</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@roofmonster.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(801)-726-1717</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Orem UT</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>80</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>residential roofing company Orem UT</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-23 19:57 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-23.xlsx
+++ b/output/leads_2026-10-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1043,6 +1043,62 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Roofer | Cambridge, MA | New Horizon Home Experts</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>newhorizonhomeexperts.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.newhorizonhomeexperts.com/contact/roofer-service-area/cambridge-ma</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>info@newhorizonhomeexperts.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(774) 274-6626</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Cambridge MA</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>roofer Cambridge MA</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-23 19:58 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-23.xlsx
+++ b/output/leads_2026-10-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1064,7 +1064,6 @@
           <t>https://www.newhorizonhomeexperts.com/contact/roofer-service-area/cambridge-ma</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>info@newhorizonhomeexperts.com</t>
@@ -1094,6 +1093,62 @@
         </is>
       </c>
       <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation in Federal Way | Eatonville Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>eatonvilleheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.eatonvilleheatingandcooling.com/heat-pump/heat-pump-installation-federal-way-wa</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>admin@eatonvilleheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(253) 406-5072</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Federal Way WA</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>heat pump installation Federal Way WA</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-23 20:00 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-23.xlsx
+++ b/output/leads_2026-10-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1119,7 +1119,6 @@
           <t>https://www.eatonvilleheatingandcooling.com/heat-pump/heat-pump-installation-federal-way-wa</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>admin@eatonvilleheatingandcooling.com</t>
@@ -1149,6 +1148,122 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Bill's Comfort Systems</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>billscomfortsystems.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.billscomfortsystems.com/hvac-company-ogden-ut-heating-cooling-services</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Home Comfort</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>service@billscomfortsystems.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(801) 544-4261</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Ogden UT</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>98</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>heating and cooling company Ogden UT</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Reliable HVAC Experts | Iowa City, IA | Davis Heating and Air</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>davisheatingandairic.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.davisheatingandairic.com/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>info@davisheatingandairic.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>319-351-0054</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Iowa City IA</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>heating and cooling company Iowa City IA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-23 20:13 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-23.xlsx
+++ b/output/leads_2026-10-23.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1234,7 +1234,6 @@
           <t>https://www.davisheatingandairic.com/</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>info@davisheatingandairic.com</t>
@@ -1264,6 +1263,122 @@
         </is>
       </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Comfortzone</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>comfortzonenm.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.comfortzonenm.com/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>shane@comfortzonenm.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>505-577-5150</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Santa Fe NM</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>HVAC contractor Santa Fe NM</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Cathedral Roofing Innovations</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>cathedralroofingflorida.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.cathedralroofingflorida.com/services/roof-repair/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Message From</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>hello@cathedralroofingflorida.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(239) 244-8822</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Naples FL</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>90</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>roof repair company Naples FL</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>2026-10-23</t>
         </is>

</xml_diff>